<commit_message>
Fill handler coordinates from FRS, rebuild panels
</commit_message>
<xml_diff>
--- a/output/panels/summary/BR_PANEL_2015_2023_Summary.xlsx
+++ b/output/panels/summary/BR_PANEL_2015_2023_Summary.xlsx
@@ -582,25 +582,25 @@
         </is>
       </c>
       <c r="B7">
-        <v>11476</v>
+        <v>25407</v>
       </c>
       <c r="C7">
-        <v>57.8</v>
+        <v>6.6</v>
       </c>
       <c r="D7">
         <v>13.4196</v>
       </c>
       <c r="E7">
-        <v>29.6754</v>
+        <v>29.7116</v>
       </c>
       <c r="F7">
-        <v>39.6741</v>
+        <v>39.6381</v>
       </c>
       <c r="G7">
-        <v>38.2385</v>
+        <v>38.2684</v>
       </c>
       <c r="H7">
-        <v>44.9598</v>
+        <v>44.9018</v>
       </c>
       <c r="I7">
         <v>70.3109</v>
@@ -613,25 +613,25 @@
         </is>
       </c>
       <c r="B8">
-        <v>11476</v>
+        <v>25407</v>
       </c>
       <c r="C8">
-        <v>57.8</v>
+        <v>6.6</v>
       </c>
       <c r="D8">
         <v>-158.1138</v>
       </c>
       <c r="E8">
-        <v>-121.7838</v>
+        <v>-121.4004</v>
       </c>
       <c r="F8">
-        <v>-86.489</v>
+        <v>-86.8206</v>
       </c>
       <c r="G8">
-        <v>-89.8639</v>
+        <v>-89.9122</v>
       </c>
       <c r="H8">
-        <v>-72.283</v>
+        <v>-72.1815</v>
       </c>
       <c r="I8">
         <v>144.6737</v>
@@ -3005,10 +3005,10 @@
         </is>
       </c>
       <c r="C131">
-        <v>26907</v>
+        <v>26846</v>
       </c>
       <c r="D131">
-        <v>98.92</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="132">
@@ -3023,10 +3023,10 @@
         </is>
       </c>
       <c r="C132">
-        <v>164</v>
+        <v>207</v>
       </c>
       <c r="D132">
-        <v>0.6</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="133">
@@ -3041,10 +3041,10 @@
         </is>
       </c>
       <c r="C133">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D133">
-        <v>0.26</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="134">
@@ -3059,10 +3059,10 @@
         </is>
       </c>
       <c r="C134">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D134">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="135">
@@ -3509,10 +3509,10 @@
         </is>
       </c>
       <c r="C159">
-        <v>24221</v>
+        <v>24144</v>
       </c>
       <c r="D159">
-        <v>89.05</v>
+        <v>88.76</v>
       </c>
     </row>
     <row r="160">
@@ -3527,10 +3527,10 @@
         </is>
       </c>
       <c r="C160">
-        <v>2954</v>
+        <v>3033</v>
       </c>
       <c r="D160">
-        <v>10.86</v>
+        <v>11.15</v>
       </c>
     </row>
     <row r="161">
@@ -3545,7 +3545,7 @@
         </is>
       </c>
       <c r="C161">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D161">
         <v>0.06</v>

</xml_diff>